<commit_message>
Update Leads_Sample with user provided test emails
</commit_message>
<xml_diff>
--- a/Leads_Sample.xlsx
+++ b/Leads_Sample.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,17 +441,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>John Doe</t>
+          <t>Chaitanya Sonaje</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>TechCorp</t>
+          <t>Tech Solutions</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>john.doe@example.com</t>
+          <t>chaitanyasonaje205@gmail.com</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -463,20 +463,86 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Jane Smith</t>
+          <t>Devendra Sonaje</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>InnovateInc</t>
+          <t>Dev Systems</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>jane.smith@example.com</t>
+          <t>devendrasonaje0205@gmail.com</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Kalpana Sonaje</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>K Enterprises</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>kalpanasonaje0205@gmail.com</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Chaitanya S</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Global AI</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>sonajechaitanya0205@gmail.com</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Dip Sonaje</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Dip Innovations</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>sonajedip@gmail.com</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>

</xml_diff>